<commit_message>
Sync Product Mapping: full tier/region coverage achieved
- Add Pingus to tier sheet
- Add new tiers: 'Napa (not cult wine)' (43 producers) and
  'Blue-chip Burgundy Producer' (15 producers)
- Result: 0 untiered, 0 unmapped region across all 184 producers

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Product Mapping - Copy.xlsx
+++ b/Producer - Product Mapping - Copy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://grandcruliquidassetscom-my.sharepoint.com/personal/chang_grandcruliquidassets_com/Documents/Desktop/Email campaign dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="562" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A28E9E9C-8F55-42A5-A8E2-0FC99124C128}"/>
+  <xr:revisionPtr revIDLastSave="564" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13905A01-BF65-47DD-AA69-C75B9936232F}"/>
   <bookViews>
-    <workbookView xWindow="47895" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="47895" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Producer - Tier" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="292">
   <si>
     <t>First Growth Producers - Flagship</t>
   </si>
@@ -51,7 +51,7 @@
     <t>Napa (not cult wine)</t>
   </si>
   <si>
-    <t>Super Tuscan Producers&amp; Others (I need to research these myself)</t>
+    <t>Super Tuscan Producers&amp; Others</t>
   </si>
   <si>
     <t>Second Label</t>
@@ -505,6 +505,9 @@
   </si>
   <si>
     <t>Tusk</t>
+  </si>
+  <si>
+    <t>Pingus</t>
   </si>
   <si>
     <t>Durfort Vivens</t>
@@ -2002,160 +2005,163 @@
         <v>153</v>
       </c>
     </row>
-    <row r="33" spans="3:4">
+    <row r="33" spans="3:5">
       <c r="C33" t="s">
         <v>154</v>
       </c>
       <c r="D33" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="34" spans="3:4">
+      <c r="E33" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="34" spans="3:5">
       <c r="C34" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D34" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="35" spans="3:4">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="35" spans="3:5">
       <c r="C35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D35" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="36" spans="3:4">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="36" spans="3:5">
       <c r="C36" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D36" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="37" spans="3:4">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="37" spans="3:5">
       <c r="C37" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D37" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="38" spans="3:4">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="38" spans="3:5">
       <c r="C38" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D38" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="39" spans="3:4">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="39" spans="3:5">
       <c r="C39" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D39" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="40" spans="3:4">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="40" spans="3:5">
       <c r="C40" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D40" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="41" spans="3:4">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="41" spans="3:5">
       <c r="C41" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D41" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="42" spans="3:4">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="42" spans="3:5">
       <c r="C42" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D42" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="43" spans="3:4">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="43" spans="3:5">
       <c r="C43" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D43" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="44" spans="3:4">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="44" spans="3:5">
       <c r="C44" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D44" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="45" spans="3:4">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="45" spans="3:5">
       <c r="C45" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="46" spans="3:4">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="46" spans="3:5">
       <c r="C46" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="47" spans="3:4">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="47" spans="3:5">
       <c r="C47" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="48" spans="3:4">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="48" spans="3:5">
       <c r="C48" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="49" spans="3:3">
       <c r="C49" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="50" spans="3:3">
       <c r="C50" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="51" spans="3:3">
       <c r="C51" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="52" spans="3:3">
       <c r="C52" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="53" spans="3:3" ht="15" customHeight="1">
       <c r="C53" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="54" spans="3:3" ht="15" customHeight="1">
       <c r="C54" s="7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="55" spans="3:3" ht="15" customHeight="1">
       <c r="C55" s="9" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="56" spans="3:3" ht="15" customHeight="1">
       <c r="C56" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -2181,58 +2187,58 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
       <c r="D1" s="13"/>
       <c r="E1" s="18" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F1" s="19"/>
       <c r="G1" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="31.5" customHeight="1">
       <c r="A2" s="16" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B2" s="16"/>
       <c r="C2" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F2" s="21" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.6">
       <c r="A3" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C3" s="17"/>
       <c r="D3" s="15"/>
@@ -2244,16 +2250,16 @@
     </row>
     <row r="4" spans="1:9" ht="15">
       <c r="A4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B4" t="s">
         <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E4" t="s">
         <v>8</v>
@@ -2263,27 +2269,27 @@
         <v>153</v>
       </c>
       <c r="H4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15">
       <c r="A5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B5" t="s">
         <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
@@ -2291,12 +2297,12 @@
         <v>147</v>
       </c>
       <c r="I5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15">
       <c r="A6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B6" t="s">
         <v>108</v>
@@ -2305,15 +2311,15 @@
         <v>69</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
       <c r="H6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I6" t="s">
         <v>18</v>
@@ -2321,16 +2327,16 @@
     </row>
     <row r="7" spans="1:9" ht="15">
       <c r="A7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B7" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E7" t="s">
         <v>29</v>
@@ -2344,16 +2350,16 @@
     </row>
     <row r="8" spans="1:9" ht="15">
       <c r="A8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E8" t="s">
         <v>36</v>
@@ -2367,16 +2373,16 @@
     </row>
     <row r="9" spans="1:9" ht="15">
       <c r="A9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C9" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E9" t="s">
         <v>43</v>
@@ -2387,19 +2393,19 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E10" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="I10" t="s">
         <v>46</v>
@@ -2413,10 +2419,10 @@
         <v>109</v>
       </c>
       <c r="C11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D11" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E11" t="s">
         <v>57</v>
@@ -2430,7 +2436,7 @@
         <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C12" t="s">
         <v>27</v>
@@ -2447,7 +2453,7 @@
     </row>
     <row r="13" spans="1:9" ht="15">
       <c r="A13" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B13" t="s">
         <v>63</v>
@@ -2467,7 +2473,7 @@
         <v>120</v>
       </c>
       <c r="B14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C14" t="s">
         <v>41</v>
@@ -2481,7 +2487,7 @@
     </row>
     <row r="15" spans="1:9" ht="15">
       <c r="A15" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B15" t="s">
         <v>87</v>
@@ -2498,10 +2504,10 @@
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B16" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C16" t="s">
         <v>55</v>
@@ -2532,16 +2538,16 @@
     </row>
     <row r="18" spans="1:9" ht="15">
       <c r="A18" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B18" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C18" t="s">
         <v>75</v>
       </c>
       <c r="E18" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I18" t="s">
         <v>94</v>
@@ -2549,10 +2555,10 @@
     </row>
     <row r="19" spans="1:9" ht="15">
       <c r="A19" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B19" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C19" t="s">
         <v>81</v>
@@ -2566,16 +2572,16 @@
     </row>
     <row r="20" spans="1:9" ht="15">
       <c r="A20" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B20" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C20" t="s">
         <v>86</v>
       </c>
       <c r="E20" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="I20" t="s">
         <v>103</v>
@@ -2583,13 +2589,13 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B21" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C21" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>74</v>
@@ -2600,10 +2606,10 @@
     </row>
     <row r="22" spans="1:9" ht="15">
       <c r="A22" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B22" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C22" t="s">
         <v>96</v>
@@ -2617,16 +2623,16 @@
     </row>
     <row r="23" spans="1:9" ht="15">
       <c r="A23" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B23" t="s">
         <v>127</v>
       </c>
       <c r="C23" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I23" t="s">
         <v>114</v>
@@ -2634,24 +2640,24 @@
     </row>
     <row r="24" spans="1:9" ht="15">
       <c r="A24" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B24" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E24" t="s">
         <v>66</v>
       </c>
       <c r="I24" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="15">
       <c r="A25" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B25" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E25" t="s">
         <v>72</v>
@@ -2662,10 +2668,10 @@
     </row>
     <row r="26" spans="1:9" ht="15">
       <c r="A26" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B26" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E26" t="s">
         <v>78</v>
@@ -2679,7 +2685,7 @@
         <v>9</v>
       </c>
       <c r="B27" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E27" t="s">
         <v>83</v>
@@ -2690,10 +2696,10 @@
     </row>
     <row r="28" spans="1:9" ht="15">
       <c r="A28" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B28" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E28" t="s">
         <v>88</v>
@@ -2707,7 +2713,7 @@
         <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E29" t="s">
         <v>93</v>
@@ -2718,7 +2724,7 @@
     </row>
     <row r="30" spans="1:9" ht="15">
       <c r="A30" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B30" t="s">
         <v>101</v>
@@ -2735,7 +2741,7 @@
         <v>71</v>
       </c>
       <c r="B31" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E31" t="s">
         <v>102</v>
@@ -2746,10 +2752,10 @@
     </row>
     <row r="32" spans="1:9" ht="15">
       <c r="A32" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B32" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E32" t="s">
         <v>106</v>
@@ -2763,7 +2769,7 @@
         <v>16</v>
       </c>
       <c r="B33" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E33" t="s">
         <v>110</v>
@@ -2777,7 +2783,7 @@
         <v>116</v>
       </c>
       <c r="B34" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E34" t="s">
         <v>113</v>
@@ -2785,13 +2791,13 @@
     </row>
     <row r="35" spans="1:9" ht="15">
       <c r="A35" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B35" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E35" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="15">
@@ -2807,13 +2813,13 @@
     </row>
     <row r="37" spans="1:9" ht="15">
       <c r="A37" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B37" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E37" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="15">
@@ -2821,7 +2827,7 @@
         <v>145</v>
       </c>
       <c r="B38" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E38" t="s">
         <v>121</v>
@@ -2829,10 +2835,10 @@
     </row>
     <row r="39" spans="1:9" ht="15">
       <c r="A39" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B39" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E39" t="s">
         <v>125</v>
@@ -2840,13 +2846,13 @@
     </row>
     <row r="40" spans="1:9" ht="15">
       <c r="A40" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B40" t="s">
         <v>42</v>
       </c>
       <c r="E40" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="15">
@@ -2854,7 +2860,7 @@
         <v>139</v>
       </c>
       <c r="B41" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E41" t="s">
         <v>129</v>
@@ -2862,21 +2868,21 @@
     </row>
     <row r="42" spans="1:9" ht="15">
       <c r="A42" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B42" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E42" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="15">
       <c r="A43" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B43" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E43" t="s">
         <v>134</v>
@@ -2884,10 +2890,10 @@
     </row>
     <row r="44" spans="1:9">
       <c r="A44" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B44" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E44" t="s">
         <v>137</v>
@@ -2895,10 +2901,10 @@
     </row>
     <row r="45" spans="1:9" ht="15">
       <c r="A45" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B45" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E45" t="s">
         <v>140</v>
@@ -2917,7 +2923,7 @@
     </row>
     <row r="47" spans="1:9" ht="15">
       <c r="A47" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B47" t="s">
         <v>119</v>
@@ -2931,21 +2937,21 @@
         <v>151</v>
       </c>
       <c r="B48" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E48" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="15">
       <c r="A49" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B49" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E49" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="15">
@@ -2953,43 +2959,43 @@
         <v>154</v>
       </c>
       <c r="B50" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E50" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="15">
       <c r="A51" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B51" s="8" t="s">
         <v>124</v>
       </c>
       <c r="E51" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="15">
       <c r="A52" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B52" t="s">
         <v>108</v>
       </c>
       <c r="E52" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="15">
       <c r="A53" s="8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B53" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E53" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="15">
@@ -3016,18 +3022,18 @@
     </row>
     <row r="56" spans="1:5" ht="15">
       <c r="A56" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B56" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E56" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="15">
       <c r="A57" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B57" t="s">
         <v>119</v>
@@ -3038,29 +3044,29 @@
     </row>
     <row r="58" spans="1:5" ht="15">
       <c r="A58" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B58" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E58" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="15">
       <c r="A59" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B59" t="s">
         <v>97</v>
       </c>
       <c r="E59" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="15">
       <c r="A60" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B60" t="s">
         <v>40</v>
@@ -3071,7 +3077,7 @@
     </row>
     <row r="61" spans="1:5" ht="15">
       <c r="A61" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E61" t="s">
         <v>15</v>
@@ -3079,7 +3085,7 @@
     </row>
     <row r="62" spans="1:5" ht="15">
       <c r="A62" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E62" t="s">
         <v>12</v>
@@ -3087,7 +3093,7 @@
     </row>
     <row r="63" spans="1:5" ht="15">
       <c r="A63" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E63" t="s">
         <v>24</v>
@@ -3095,20 +3101,20 @@
     </row>
     <row r="64" spans="1:5" ht="15">
       <c r="A64" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E64" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="65" spans="1:1" ht="15">
       <c r="A65" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="66" spans="1:1" ht="15">
       <c r="A66" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="67" spans="1:1" ht="15">

</xml_diff>

<commit_message>
Add tier/region for Nine Suns, Clos Erasmus, Rayas
- Nine Suns    -> Napa (not cult wine)          / US / California
- Clos Erasmus -> Super Tuscan Producers& Others / Spain
- Rayas        -> Second Label                  / France / Other France

Meursault (Mersault White burgundy) still has no tier/region assigned.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Product Mapping - Copy.xlsx
+++ b/Producer - Product Mapping - Copy.xlsx
@@ -1420,6 +1420,11 @@
           <t>Gaja</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Rayas</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15.5" customHeight="1">
       <c r="C26" s="2" t="inlineStr">
@@ -1619,6 +1624,11 @@
           <t>Morlet</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Clos Erasmus</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="14.5" customHeight="1">
       <c r="C38" t="inlineStr">
@@ -1744,6 +1754,11 @@
       <c r="C48" t="inlineStr">
         <is>
           <t>La Mission Haut Brion</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Nine Suns</t>
         </is>
       </c>
     </row>
@@ -2098,7 +2113,11 @@
       </c>
       <c r="F7" s="8" t="n"/>
       <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Clos Erasmus</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>Solaia</t>
@@ -2348,6 +2367,11 @@
           <t>Domaine Ponsot</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Rayas</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>Promontory</t>
@@ -3362,6 +3386,11 @@
       <c r="A68" t="inlineStr">
         <is>
           <t>Carruades de Lafite</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Nine Suns</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Move Vega Sicilia to Super Second Producers tier
Was under Super Tuscan Producers & Others. Region stays Spain (unchanged).
Peter Michael confirmed already correct: Napa (not cult wine) / US California.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producer - Product Mapping - Copy.xlsx
+++ b/Producer - Product Mapping - Copy.xlsx
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1505,11 +1505,6 @@
           <t>Marcassin</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Vega Sicilia</t>
-        </is>
-      </c>
     </row>
     <row r="31" ht="14.5" customHeight="1">
       <c r="C31" t="inlineStr">
@@ -1843,6 +1838,13 @@
       <c r="C60" t="inlineStr">
         <is>
           <t>Larcis Ducasse</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Vega Sicilia</t>
         </is>
       </c>
     </row>

</xml_diff>